<commit_message>
data: refresh sku_master + W22 WM raw inventory
Master grew from 85 KB to 172 KB — adds recent ASINs that W18-W22
inventory rows depend on. Pushing this unblocks the weekly-sync
workflow: runner was rebuilding inventory_model_snapshot with the stale
May 28 master, dropping all unresolved rows, and tripping the audit's
fail-loud cross-route checks.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/inventory/Week 22/White_Mulberry/Inventory Snapshot.xlsx
+++ b/data/raw/inventory/Week 22/White_Mulberry/Inventory Snapshot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 22\White_Mulberry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA2F95E8-261C-40A1-BFFC-1DC735184268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7164F237-61A1-4D50-8B38-A0B5E09AD8C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D49B0F4C-5F9E-467E-8AD9-9E638F42404F}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="128">
   <si>
     <t>SKU</t>
   </si>
@@ -345,82 +345,85 @@
     <t>B0FN4HDBN5</t>
   </si>
   <si>
+    <t>WM-MH05P-BK</t>
+  </si>
+  <si>
+    <t>WM-SMD09-WH</t>
+  </si>
+  <si>
+    <t>WM-SE08-CF</t>
+  </si>
+  <si>
+    <t>WM-SE08-WH</t>
+  </si>
+  <si>
+    <t>6780-4679-WHT-SIOC</t>
+  </si>
+  <si>
+    <t>WM-LOD-IN</t>
+  </si>
+  <si>
+    <t>WM-LODN-BK</t>
+  </si>
+  <si>
+    <t>MS2ML</t>
+  </si>
+  <si>
+    <t>VLMS1ML</t>
+  </si>
+  <si>
+    <t>WM-MODL-WH</t>
+  </si>
+  <si>
+    <t>POS2M</t>
+  </si>
+  <si>
+    <t>POS2MK</t>
+  </si>
+  <si>
+    <t>POS BRACKET</t>
+  </si>
+  <si>
+    <t>TVCF1ML</t>
+  </si>
+  <si>
+    <t>HDMSP1ML</t>
+  </si>
+  <si>
+    <t>HDGS1ML</t>
+  </si>
+  <si>
+    <t>TVCT1ML</t>
+  </si>
+  <si>
+    <t>TVMF1ML</t>
+  </si>
+  <si>
+    <t>TVLF1ML</t>
+  </si>
+  <si>
+    <t>TVFM1ML</t>
+  </si>
+  <si>
+    <t>B2B - AMPM</t>
+  </si>
+  <si>
+    <t>TC777 Pro</t>
+  </si>
+  <si>
+    <t>YNT</t>
+  </si>
+  <si>
+    <t>Open Order</t>
+  </si>
+  <si>
+    <t>Pipeline</t>
+  </si>
+  <si>
+    <t>FBK79790</t>
+  </si>
+  <si>
     <t>B0FN4GJ9S1</t>
-  </si>
-  <si>
-    <t>WM-MH05P-BK</t>
-  </si>
-  <si>
-    <t>WM-SMD09-WH</t>
-  </si>
-  <si>
-    <t>WM-SE08-CF</t>
-  </si>
-  <si>
-    <t>WM-SE08-WH</t>
-  </si>
-  <si>
-    <t>6780-4679-WHT-SIOC</t>
-  </si>
-  <si>
-    <t>WM-LOD-IN</t>
-  </si>
-  <si>
-    <t>WM-LODN-BK</t>
-  </si>
-  <si>
-    <t>MS2ML</t>
-  </si>
-  <si>
-    <t>VLMS1ML</t>
-  </si>
-  <si>
-    <t>WM-MODL-WH</t>
-  </si>
-  <si>
-    <t>POS2M</t>
-  </si>
-  <si>
-    <t>POS2MK</t>
-  </si>
-  <si>
-    <t>POS BRACKET</t>
-  </si>
-  <si>
-    <t>TVCF1ML</t>
-  </si>
-  <si>
-    <t>HDMSP1ML</t>
-  </si>
-  <si>
-    <t>HDGS1ML</t>
-  </si>
-  <si>
-    <t>TVCT1ML</t>
-  </si>
-  <si>
-    <t>TVMF1ML</t>
-  </si>
-  <si>
-    <t>TVLF1ML</t>
-  </si>
-  <si>
-    <t>TVFM1ML</t>
-  </si>
-  <si>
-    <t>B2B - AMPM</t>
-  </si>
-  <si>
-    <t>TC777 Pro</t>
-  </si>
-  <si>
-    <t>YNT</t>
-  </si>
-  <si>
-    <t>Open Order</t>
-  </si>
-  <si>
-    <t>Pipeline</t>
   </si>
 </sst>
 </file>
@@ -540,7 +543,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -573,6 +576,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
@@ -6124,7 +6130,7 @@
         <v>95</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I41" s="4">
         <v>1</v>
@@ -6144,7 +6150,7 @@
         <v>95</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I42" s="4">
         <v>15</v>
@@ -6164,7 +6170,7 @@
         <v>95</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I43" s="4">
         <v>13</v>
@@ -6184,7 +6190,7 @@
         <v>95</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I44" s="4">
         <v>23</v>
@@ -6204,7 +6210,7 @@
         <v>95</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I45" s="4">
         <v>1</v>
@@ -6224,7 +6230,7 @@
         <v>95</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I46" s="4">
         <v>1</v>
@@ -6284,7 +6290,7 @@
         <v>95</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I49" s="4">
         <v>15</v>
@@ -6324,7 +6330,7 @@
         <v>95</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I51" s="4">
         <v>4</v>
@@ -6344,7 +6350,7 @@
         <v>95</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I52" s="4">
         <v>311</v>
@@ -6404,7 +6410,7 @@
         <v>95</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I55" s="4">
         <v>12</v>
@@ -6424,7 +6430,7 @@
         <v>95</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I56" s="4">
         <v>18</v>
@@ -6444,7 +6450,7 @@
         <v>95</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I57" s="4">
         <v>18</v>
@@ -6464,7 +6470,7 @@
         <v>95</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I58" s="4">
         <v>112</v>
@@ -6484,7 +6490,7 @@
         <v>95</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I59" s="4">
         <v>638</v>
@@ -6504,7 +6510,7 @@
         <v>95</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I60" s="4">
         <v>15</v>
@@ -6524,7 +6530,7 @@
         <v>95</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I61" s="4">
         <v>6</v>
@@ -6544,7 +6550,7 @@
         <v>95</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I62" s="4">
         <v>296</v>
@@ -6554,17 +6560,17 @@
       </c>
     </row>
     <row r="63" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>101</v>
+      <c r="A63" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="B63" t="s">
+        <v>127</v>
       </c>
       <c r="C63" t="s">
         <v>95</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I63" s="4">
         <v>655</v>
@@ -6584,7 +6590,7 @@
         <v>95</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I64" s="4">
         <v>610</v>
@@ -6604,13 +6610,13 @@
         <v>95</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I65" s="4">
         <v>4</v>
       </c>
       <c r="J65" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="66" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -6630,7 +6636,7 @@
         <v>2</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="67" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -6644,13 +6650,13 @@
         <v>95</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I67" s="4">
         <v>3</v>
       </c>
       <c r="J67" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="68" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -6670,7 +6676,7 @@
         <v>4</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="69" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -6690,7 +6696,7 @@
         <v>5</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="70" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -6711,7 +6717,7 @@
         <v>5</v>
       </c>
       <c r="J70" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K70" s="7"/>
     </row>
@@ -6733,7 +6739,7 @@
         <v>4</v>
       </c>
       <c r="J71" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K71" s="7"/>
     </row>
@@ -6749,13 +6755,13 @@
         <v>95</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I72" s="8">
         <v>3</v>
       </c>
       <c r="J72" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K72" s="7"/>
     </row>
@@ -6777,7 +6783,7 @@
         <v>2</v>
       </c>
       <c r="J73" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K73" s="7"/>
     </row>
@@ -6798,7 +6804,7 @@
         <v>1000</v>
       </c>
       <c r="J74" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K74" s="9"/>
     </row>
@@ -6813,13 +6819,13 @@
         <v>95</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I75" s="11">
         <v>1000</v>
       </c>
       <c r="J75" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K75" s="9"/>
     </row>
@@ -6840,12 +6846,11 @@
         <v>500</v>
       </c>
       <c r="J76" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K76" s="9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L76" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="A41:A64">
     <cfRule type="duplicateValues" dxfId="34" priority="2559"/>

</xml_diff>